<commit_message>
AI soạn quy trình
</commit_message>
<xml_diff>
--- a/hop/notes.xlsx
+++ b/hop/notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ThanhVu\kpht\KPHT_PMM\hop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594E7AC9-2989-4FE7-9B57-B8B7949295A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246BB080-D0A7-4BB6-856F-77537CC83C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2055" yWindow="1485" windowWidth="17580" windowHeight="13995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>